<commit_message>
Restaurant: route to its own CMA, table-based covers, wages counted once
- refine_industry(): a new project saved as hospitality whose sub-industry/title
  describe a restaurant (and no lodging) is stored as Food & Beverage / Restaurant,
  so it gets the restaurant workbook instead of room-nights x ARR.
- CMA_Restaurant.xlsx: Assumptions!C16 = E16*F16*G16*H16*I16 (tables x seats x
  table turns x occupancy x days). reconcile_covers_drivers back-solves turns so
  the drivers equal the settled covers; fill_template never overwrites C16.
- _monthly_fixed_total counted the shared E32xF32 wage pair once per industry
  template (10x), so reconcile_scale inflated volumes on every volume-price
  template (60,000 restaurant covers came out as 10 lakh).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/restaurant_cma/CMA_Restaurant.xlsx
+++ b/templates/restaurant_cma/CMA_Restaurant.xlsx
@@ -10405,13 +10405,35 @@
           <t>Covers served (Year 1)</t>
         </is>
       </c>
-      <c r="C16" s="121" t="n"/>
+      <c r="C16" s="121">
+        <f>E16*F16*G16*H16*I16</f>
+        <v/>
+      </c>
       <c r="D16" s="283" t="inlineStr">
         <is>
           <t>units p.a.</t>
         </is>
       </c>
-      <c r="H16" s="118" t="n"/>
+      <c r="E16" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="125" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="81" t="inlineStr">
+        <is>
+          <t>(E16 tables × F16 seats/table × G16 table turns/day × H16 occupancy × I16 days open p.a.)</t>
+        </is>
+      </c>
       <c r="S16" s="81" t="inlineStr">
         <is>
           <t>Transportation &amp; Logistics</t>

</xml_diff>